<commit_message>
Added responsive design using Claude
</commit_message>
<xml_diff>
--- a/database/students.xlsx
+++ b/database/students.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\face_attendance_system\database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Face-Recognition-Attendance-System\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49E595E0-C498-4EFD-A7D6-8F5F9FD46D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E6DD46-2646-4ED7-B3D1-2D0C5F83A288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3900" yWindow="3390" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="81">
   <si>
     <t>name</t>
   </si>
@@ -262,6 +262,12 @@
   </si>
   <si>
     <t>alnoman.8363@gmail.com</t>
+  </si>
+  <si>
+    <t>md.tonmoyratul@gmail.com</t>
+  </si>
+  <si>
+    <t>ibrahimhossain3669@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -911,7 +917,9 @@
       <c r="E13" s="6">
         <v>230525</v>
       </c>
-      <c r="F13" s="9"/>
+      <c r="F13" s="12" t="s">
+        <v>80</v>
+      </c>
       <c r="G13" s="5" t="s">
         <v>9</v>
       </c>
@@ -1001,7 +1009,9 @@
       <c r="E17" s="5">
         <v>230530</v>
       </c>
-      <c r="F17" s="9"/>
+      <c r="F17" s="11" t="s">
+        <v>79</v>
+      </c>
       <c r="G17" s="5" t="s">
         <v>9</v>
       </c>
@@ -2712,6 +2722,8 @@
     <hyperlink ref="F18" r:id="rId40" xr:uid="{EBAA85DE-C558-4142-836A-A9E2B8ECBCCE}"/>
     <hyperlink ref="F11" r:id="rId41" xr:uid="{CCEBB030-3363-47F4-B381-BB5741154D20}"/>
     <hyperlink ref="F20" r:id="rId42" xr:uid="{C1FE2B22-4057-4486-97FC-397C12F3A7E9}"/>
+    <hyperlink ref="F17" r:id="rId43" xr:uid="{E6291E75-B67C-4384-90C8-9CE14AC6EC5C}"/>
+    <hyperlink ref="F13" r:id="rId44" xr:uid="{0DF3BBA1-5AA2-4C98-A85A-D7568E6809C2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>

</xml_diff>